<commit_message>
Casos de tesis swap: topes de generacion y BESS en 10 (g_max, h_max) donde estan permitidos
En la practica quedan libres. Zona centro (caso 6) se cambia al terminar su corrida con
tope 2, que quedaba en el limite de solar (2,0 modulos); se relanza con tope 10.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Tesis_final/Mina_modelo/Produccion_base/zona_centro_v4/05C/RED_GEN_BESS/elmo_data.xlsx
+++ b/data/Tesis_final/Mina_modelo/Produccion_base/zona_centro_v4/05C/RED_GEN_BESS/elmo_data.xlsx
@@ -1797,7 +1797,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
     <col width="13.5546875" bestFit="1" customWidth="1" style="6" min="1" max="1"/>
@@ -3170,414 +3170,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
-    <row r="220"/>
-    <row r="221"/>
-    <row r="222"/>
-    <row r="223"/>
-    <row r="224"/>
-    <row r="225"/>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
-    <row r="260"/>
-    <row r="261"/>
-    <row r="262"/>
-    <row r="263"/>
-    <row r="264"/>
-    <row r="265"/>
-    <row r="266"/>
-    <row r="267"/>
-    <row r="268"/>
-    <row r="269"/>
-    <row r="270"/>
-    <row r="271"/>
-    <row r="272"/>
-    <row r="273"/>
-    <row r="274"/>
-    <row r="275"/>
-    <row r="276"/>
-    <row r="277"/>
-    <row r="278"/>
-    <row r="279"/>
-    <row r="280"/>
-    <row r="281"/>
-    <row r="282"/>
-    <row r="283"/>
-    <row r="284"/>
-    <row r="285"/>
-    <row r="286"/>
-    <row r="287"/>
-    <row r="288"/>
-    <row r="289"/>
-    <row r="290"/>
-    <row r="291"/>
-    <row r="292"/>
-    <row r="293"/>
-    <row r="294"/>
-    <row r="295"/>
-    <row r="296"/>
-    <row r="297"/>
-    <row r="298"/>
-    <row r="299"/>
-    <row r="300"/>
-    <row r="301"/>
-    <row r="302"/>
-    <row r="303"/>
-    <row r="304"/>
-    <row r="305"/>
-    <row r="306"/>
-    <row r="307"/>
-    <row r="308"/>
-    <row r="309"/>
-    <row r="310"/>
-    <row r="311"/>
-    <row r="312"/>
-    <row r="313"/>
-    <row r="314"/>
-    <row r="315"/>
-    <row r="316"/>
-    <row r="317"/>
-    <row r="318"/>
-    <row r="319"/>
-    <row r="320"/>
-    <row r="321"/>
-    <row r="322"/>
-    <row r="323"/>
-    <row r="324"/>
-    <row r="325"/>
-    <row r="326"/>
-    <row r="327"/>
-    <row r="328"/>
-    <row r="329"/>
-    <row r="330"/>
-    <row r="331"/>
-    <row r="332"/>
-    <row r="333"/>
-    <row r="334"/>
-    <row r="335"/>
-    <row r="336"/>
-    <row r="337"/>
-    <row r="338"/>
-    <row r="339"/>
-    <row r="340"/>
-    <row r="341"/>
-    <row r="342"/>
-    <row r="343"/>
-    <row r="344"/>
-    <row r="345"/>
-    <row r="346"/>
-    <row r="347"/>
-    <row r="348"/>
-    <row r="349"/>
-    <row r="350"/>
-    <row r="351"/>
-    <row r="352"/>
-    <row r="353"/>
-    <row r="354"/>
-    <row r="355"/>
-    <row r="356"/>
-    <row r="357"/>
-    <row r="358"/>
-    <row r="359"/>
-    <row r="360"/>
-    <row r="361"/>
-    <row r="362"/>
-    <row r="363"/>
-    <row r="364"/>
-    <row r="365"/>
-    <row r="366"/>
-    <row r="367"/>
-    <row r="368"/>
-    <row r="369"/>
-    <row r="370"/>
-    <row r="371"/>
-    <row r="372"/>
-    <row r="373"/>
-    <row r="374"/>
-    <row r="375"/>
-    <row r="376"/>
-    <row r="377"/>
-    <row r="378"/>
-    <row r="379"/>
-    <row r="380"/>
-    <row r="381"/>
-    <row r="382"/>
-    <row r="383"/>
-    <row r="384"/>
-    <row r="385"/>
-    <row r="386"/>
-    <row r="387"/>
-    <row r="388"/>
-    <row r="389"/>
-    <row r="390"/>
-    <row r="391"/>
-    <row r="392"/>
-    <row r="393"/>
-    <row r="394"/>
-    <row r="395"/>
-    <row r="396"/>
-    <row r="397"/>
-    <row r="398"/>
-    <row r="399"/>
-    <row r="400"/>
-    <row r="401"/>
-    <row r="402"/>
-    <row r="403"/>
-    <row r="404"/>
-    <row r="405"/>
-    <row r="406"/>
-    <row r="407"/>
-    <row r="408"/>
-    <row r="409"/>
-    <row r="410"/>
-    <row r="411"/>
-    <row r="412"/>
-    <row r="413"/>
-    <row r="414"/>
-    <row r="415"/>
-    <row r="416"/>
-    <row r="417"/>
-    <row r="418"/>
-    <row r="419"/>
-    <row r="420"/>
-    <row r="421"/>
-    <row r="422"/>
-    <row r="423"/>
-    <row r="424"/>
-    <row r="425"/>
-    <row r="426"/>
-    <row r="427"/>
-    <row r="428"/>
-    <row r="429"/>
-    <row r="430"/>
-    <row r="431"/>
-    <row r="432"/>
-    <row r="433"/>
-    <row r="434"/>
-    <row r="435"/>
-    <row r="436"/>
-    <row r="437"/>
-    <row r="438"/>
-    <row r="439"/>
-    <row r="440"/>
-    <row r="441"/>
-    <row r="442"/>
-    <row r="443"/>
-    <row r="444"/>
-    <row r="445"/>
-    <row r="446"/>
-    <row r="447"/>
-    <row r="448"/>
-    <row r="449"/>
-    <row r="450"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3757,7 +3349,7 @@
         <v>500</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
@@ -3784,7 +3376,7 @@
         <v>500</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -3923,7 +3515,7 @@
         <v>1000</v>
       </c>
       <c r="I3" s="21" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>